<commit_message>
updated version of search words
</commit_message>
<xml_diff>
--- a/SPAS-META相关_Final.xlsx
+++ b/SPAS-META相关_Final.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="25320" windowHeight="12140" activeTab="1"/>
+    <workbookView windowWidth="25340" windowHeight="12160" activeTab="1"/>
   </bookViews>
   <sheets>
     <sheet name="zoey" sheetId="1" r:id="rId1"/>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="60" uniqueCount="47">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="64" uniqueCount="51">
   <si>
     <t>PICOS+关键词</t>
   </si>
@@ -213,6 +213,9 @@
     <t>PICOS原则：红色部分是我建议纳入检索框的模块</t>
   </si>
   <si>
+    <t>优化</t>
+  </si>
+  <si>
     <t>备注</t>
   </si>
   <si>
@@ -228,10 +231,20 @@
 OR "Women's Group"[Title/Abstract]</t>
   </si>
   <si>
+    <t>"Female" OR "Girl" OR "Woman" OR "Women's Group"</t>
+  </si>
+  <si>
     <t>检索阶段是否可以把P（female）模块从AND逻辑里去掉，从而避免漏掉那些题目摘要里没提性别但是正文里有可提取女性数据的研究。针对混合样本，若正文附录报告了按性别拆分的数据，便纳入且只提取女性亚组的效应量数据；若未报告性别拆分数据，但女性占比可辨识，便联系作者索要未发表的性别拆分数据</t>
   </si>
   <si>
     <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="宋体"/>
+        <charset val="134"/>
+        <scheme val="minor"/>
+      </rPr>
       <t>考虑检索的文献库：</t>
     </r>
     <r>
@@ -313,7 +326,15 @@
 OR "Training, Human Physical"[Title/Abstract]
 5. "Motor Activity"[Mesh]: "Activities, Motor"[Title/Abstract]
 OR "Activity, Motor"[Title/Abstract]
-OR "Motor Activities"[Title/Abstract]</t>
+OR "Motor Activities"[Title/Abstract]
+6. Others: OR "yoga"[Title/Abstract]
+OR "pilates"[Title/Abstract]
+OR "dance"[Title/Abstract]
+OR "dancing"[Title/Abstract]
+OR "fitness"[Title/Abstract]</t>
+  </si>
+  <si>
+    <t>“Sport" OR "Athletic" OR "Exercise" OR "Physical Exercise" OR "Isometric Exercise" OR "Aerobic Exercise" OR "Exercise Training" OR "Physical Activity" OR "Active Break" OR "Acute Exercise" OR "Exercise Therapy" OR "Exercise Prescription" OR "Rehabilitation Exercise" OR "Remedial Exercise" OR "Exercise Therapy" OR "Physical Activity Intervention" OR "Human Physical Conditioning" OR "Human Physical Training" OR "Motor Activity" OR "yoga" OR "pilates" OR "dance" OR "dancing" OR "fitness" OR "dance movement" OR "dance movement therapy"</t>
   </si>
   <si>
     <t>"social physique anxiety"[Title/Abstract]
@@ -324,10 +345,22 @@
 OR "SPAS-7"[Title/Abstract]</t>
   </si>
   <si>
+    <t>"social physique anxiety" OR "social physical anxiety" OR "physique anxiety" OR "Social Physique Anxiety Scale" OR "SPAS" OR "SPAS-7" OR "anxiety" OR "social anxiety" OR "physical activity and anxiety" OR "anxiety about body" OR "body image" OR "self-consciousness" OR "anxiousness"</t>
+  </si>
+  <si>
     <t>Mesh医学词库没有相关的词汇</t>
   </si>
   <si>
     <r>
+      <rPr>
+        <b/>
+        <u/>
+        <sz val="18"/>
+        <color theme="1"/>
+        <rFont val="宋体"/>
+        <charset val="134"/>
+        <scheme val="minor"/>
+      </rPr>
       <t>中文纳入标准</t>
     </r>
     <r>
@@ -627,6 +660,13 @@
       <scheme val="minor"/>
     </font>
     <font>
+      <sz val="11"/>
+      <color rgb="FFFF0000"/>
+      <name val="宋体"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
       <u/>
       <sz val="18"/>
       <color theme="1"/>
@@ -634,20 +674,25 @@
       <charset val="134"/>
       <scheme val="minor"/>
     </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FFFF0000"/>
-      <name val="宋体"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
   </fonts>
-  <fills count="33">
+  <fills count="35">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.8"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.8"/>
+        <bgColor indexed="64"/>
+      </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
@@ -1005,7 +1050,7 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="4" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="4" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
@@ -1029,16 +1074,16 @@
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="3" borderId="7" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="4" borderId="8" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="4" borderId="7" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="5" borderId="9" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="12" fillId="5" borderId="7" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="6" borderId="8" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="6" borderId="7" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="7" borderId="9" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="16" fillId="0" borderId="10" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
@@ -1047,90 +1092,93 @@
     <xf numFmtId="0" fontId="17" fillId="0" borderId="11" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="6" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="18" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="34" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="22">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -1142,26 +1190,44 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1">
       <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1">
       <alignment vertical="center"/>
@@ -1703,124 +1769,124 @@
   <dimension ref="A1:C20"/>
   <sheetFormatPr defaultColWidth="9.23076923076923" defaultRowHeight="26" outlineLevelCol="2"/>
   <cols>
-    <col min="1" max="1" width="41.0192307692308" style="10" customWidth="1"/>
-    <col min="2" max="2" width="196.442307692308" style="10" customWidth="1"/>
-    <col min="3" max="3" width="254.875" style="10" customWidth="1"/>
-    <col min="4" max="16384" width="9.23076923076923" style="10"/>
+    <col min="1" max="1" width="41.0192307692308" style="15" customWidth="1"/>
+    <col min="2" max="2" width="196.442307692308" style="15" customWidth="1"/>
+    <col min="3" max="3" width="254.875" style="15" customWidth="1"/>
+    <col min="4" max="16384" width="9.23076923076923" style="15"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:3">
-      <c r="A1" s="2" t="s">
+      <c r="A1" s="3" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="3" t="s">
+      <c r="B1" s="4" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="12" t="s">
+      <c r="C1" s="19" t="s">
         <v>2</v>
       </c>
     </row>
     <row r="2" ht="182" spans="1:3">
-      <c r="A2" s="4" t="s">
+      <c r="A2" s="6" t="s">
         <v>3</v>
       </c>
-      <c r="B2" s="5" t="s">
+      <c r="B2" s="7" t="s">
         <v>4</v>
       </c>
-      <c r="C2" s="13"/>
+      <c r="C2" s="20"/>
     </row>
     <row r="3" ht="409" customHeight="1" spans="1:3">
-      <c r="A3" s="4" t="s">
+      <c r="A3" s="6" t="s">
         <v>5</v>
       </c>
-      <c r="B3" s="5" t="s">
+      <c r="B3" s="7" t="s">
         <v>6</v>
       </c>
-      <c r="C3" s="13"/>
+      <c r="C3" s="20"/>
     </row>
     <row r="4" spans="1:3">
-      <c r="A4" s="4" t="s">
+      <c r="A4" s="6" t="s">
         <v>7</v>
       </c>
-      <c r="B4" s="3"/>
-      <c r="C4" s="13"/>
+      <c r="B4" s="4"/>
+      <c r="C4" s="20"/>
     </row>
     <row r="5" ht="78" spans="1:3">
-      <c r="A5" s="4" t="s">
+      <c r="A5" s="6" t="s">
         <v>8</v>
       </c>
-      <c r="B5" s="5" t="s">
+      <c r="B5" s="7" t="s">
         <v>9</v>
       </c>
-      <c r="C5" s="13"/>
+      <c r="C5" s="20"/>
     </row>
     <row r="6" spans="1:3">
-      <c r="A6" s="4" t="s">
+      <c r="A6" s="6" t="s">
         <v>10</v>
       </c>
-      <c r="B6" s="3"/>
-      <c r="C6" s="14"/>
+      <c r="B6" s="4"/>
+      <c r="C6" s="21"/>
     </row>
     <row r="11" ht="409" customHeight="1" spans="1:3">
-      <c r="A11" s="7" t="s">
+      <c r="A11" s="11" t="s">
         <v>11</v>
       </c>
-      <c r="B11" s="9" t="s">
+      <c r="B11" s="14" t="s">
         <v>12</v>
       </c>
-      <c r="C11" s="9" t="s">
+      <c r="C11" s="14" t="s">
         <v>13</v>
       </c>
     </row>
     <row r="14" ht="104" spans="1:3">
-      <c r="A14" s="7" t="s">
+      <c r="A14" s="11" t="s">
         <v>14</v>
       </c>
-      <c r="B14" s="9" t="s">
+      <c r="B14" s="14" t="s">
         <v>15</v>
       </c>
-      <c r="C14" s="9" t="s">
+      <c r="C14" s="14" t="s">
         <v>16</v>
       </c>
     </row>
     <row r="15" ht="104" spans="1:3">
-      <c r="A15" s="7" t="s">
+      <c r="A15" s="11" t="s">
         <v>17</v>
       </c>
-      <c r="B15" s="9" t="s">
+      <c r="B15" s="14" t="s">
         <v>18</v>
       </c>
-      <c r="C15" s="9" t="s">
+      <c r="C15" s="14" t="s">
         <v>19</v>
       </c>
     </row>
     <row r="16" ht="78" spans="1:3">
-      <c r="A16" s="7" t="s">
+      <c r="A16" s="11" t="s">
         <v>20</v>
       </c>
-      <c r="B16" s="9" t="s">
+      <c r="B16" s="14" t="s">
         <v>21</v>
       </c>
-      <c r="C16" s="9" t="s">
+      <c r="C16" s="14" t="s">
         <v>22</v>
       </c>
     </row>
     <row r="18" spans="1:3">
-      <c r="A18" s="7" t="s">
+      <c r="A18" s="11" t="s">
         <v>23</v>
       </c>
-      <c r="B18" s="11" t="s">
+      <c r="B18" s="18" t="s">
         <v>24</v>
       </c>
     </row>
     <row r="20" ht="338" spans="1:3">
-      <c r="A20" s="11" t="s">
+      <c r="A20" s="18" t="s">
         <v>25</v>
       </c>
-      <c r="B20" s="9" t="s">
+      <c r="B20" s="14" t="s">
         <v>26</v>
       </c>
-      <c r="C20" s="9" t="s">
+      <c r="C20" s="14" t="s">
         <v>27</v>
       </c>
     </row>
@@ -1836,158 +1902,183 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:E18"/>
-  <sheetFormatPr defaultColWidth="9.23076923076923" defaultRowHeight="16.8" outlineLevelCol="4"/>
+  <dimension ref="A1:F18"/>
+  <sheetFormatPr defaultColWidth="9.23076923076923" defaultRowHeight="16.8" outlineLevelCol="5"/>
   <cols>
     <col min="1" max="1" width="37.0192307692308" customWidth="1"/>
     <col min="2" max="2" width="91.3461538461538" customWidth="1"/>
-    <col min="3" max="3" width="73.9807692307692" style="1" customWidth="1"/>
-    <col min="4" max="4" width="18.2692307692308" style="1" customWidth="1"/>
-    <col min="5" max="5" width="28.2019230769231" customWidth="1"/>
+    <col min="3" max="3" width="91.3461538461538" style="1" customWidth="1"/>
+    <col min="4" max="4" width="73.9807692307692" style="2" customWidth="1"/>
+    <col min="5" max="5" width="18.2692307692308" style="2" customWidth="1"/>
+    <col min="6" max="6" width="28.2019230769231" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="57" customHeight="1" spans="1:5">
-      <c r="A1" s="2" t="s">
+    <row r="1" ht="57" customHeight="1" spans="1:6">
+      <c r="A1" s="3" t="s">
         <v>28</v>
       </c>
-      <c r="B1" s="3" t="s">
+      <c r="B1" s="4" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" s="5" t="s">
         <v>29</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" s="2" t="s">
         <v>30</v>
       </c>
-    </row>
-    <row r="2" ht="202" spans="1:5">
-      <c r="A2" s="4" t="s">
+      <c r="E1" s="2" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="2" ht="182" spans="1:6">
+      <c r="A2" s="6" t="s">
         <v>3</v>
       </c>
-      <c r="B2" s="5" t="s">
-        <v>31</v>
-      </c>
-      <c r="C2" s="1" t="s">
+      <c r="B2" s="7" t="s">
         <v>32</v>
       </c>
-      <c r="D2" s="1"/>
-      <c r="E2" s="6" t="s">
+      <c r="C2" s="8" t="s">
         <v>33</v>
       </c>
-    </row>
-    <row r="3" ht="409.5" spans="1:5">
-      <c r="A3" s="2" t="s">
+      <c r="D2" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="F2" s="9" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="3" ht="409.5" spans="1:6">
+      <c r="A3" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="B3" s="5" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="4" ht="26" spans="1:5">
-      <c r="A4" s="4" t="s">
+      <c r="B3" s="7" t="s">
+        <v>36</v>
+      </c>
+      <c r="C3" s="10" t="s">
+        <v>37</v>
+      </c>
+      <c r="D3" s="7"/>
+    </row>
+    <row r="4" ht="26" spans="1:6">
+      <c r="A4" s="6" t="s">
         <v>7</v>
       </c>
-      <c r="B4" s="3"/>
-    </row>
-    <row r="5" ht="156" spans="1:5">
-      <c r="A5" s="2" t="s">
+      <c r="B4" s="4"/>
+      <c r="C4" s="5"/>
+    </row>
+    <row r="5" ht="156" spans="1:6">
+      <c r="A5" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="B5" s="5" t="s">
-        <v>35</v>
-      </c>
-      <c r="C5" s="1" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="6" ht="26" spans="1:5">
-      <c r="A6" s="4" t="s">
+      <c r="B5" s="7" t="s">
+        <v>38</v>
+      </c>
+      <c r="C5" s="8" t="s">
+        <v>39</v>
+      </c>
+      <c r="D5" s="2" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="6" ht="26" spans="1:6">
+      <c r="A6" s="6" t="s">
         <v>10</v>
       </c>
-      <c r="B6" s="3"/>
-    </row>
-    <row r="9" ht="409" customHeight="1" spans="1:5">
-      <c r="A9" s="7" t="s">
+      <c r="B6" s="4"/>
+      <c r="C6" s="5"/>
+    </row>
+    <row r="9" ht="409" customHeight="1" spans="1:6">
+      <c r="A9" s="11" t="s">
         <v>11</v>
       </c>
-      <c r="B9" s="8" t="s">
-        <v>37</v>
-      </c>
-      <c r="C9" s="9" t="s">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="10" ht="26" spans="1:5">
-      <c r="A10" s="10"/>
-      <c r="B10" s="10"/>
-      <c r="C10" s="10"/>
-    </row>
-    <row r="11" ht="26" spans="1:5">
-      <c r="A11" s="10"/>
-      <c r="B11" s="10"/>
-      <c r="C11" s="10"/>
-    </row>
-    <row r="12" ht="260" spans="1:5">
-      <c r="A12" s="7" t="s">
+      <c r="B9" s="12" t="s">
+        <v>41</v>
+      </c>
+      <c r="C9" s="13"/>
+      <c r="D9" s="14" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="10" ht="26" spans="1:6">
+      <c r="A10" s="15"/>
+      <c r="B10" s="15"/>
+      <c r="C10" s="16"/>
+      <c r="D10" s="15"/>
+    </row>
+    <row r="11" ht="26" spans="1:6">
+      <c r="A11" s="15"/>
+      <c r="B11" s="15"/>
+      <c r="C11" s="16"/>
+      <c r="D11" s="15"/>
+    </row>
+    <row r="12" ht="260" spans="1:6">
+      <c r="A12" s="11" t="s">
         <v>14</v>
       </c>
-      <c r="B12" s="9" t="s">
-        <v>39</v>
-      </c>
-      <c r="C12" s="9" t="s">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="13" ht="260" spans="1:5">
-      <c r="A13" s="7" t="s">
+      <c r="B12" s="14" t="s">
+        <v>43</v>
+      </c>
+      <c r="C12" s="17"/>
+      <c r="D12" s="14" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="13" ht="260" spans="1:6">
+      <c r="A13" s="11" t="s">
         <v>17</v>
       </c>
-      <c r="B13" s="9" t="s">
-        <v>41</v>
-      </c>
-      <c r="C13" s="9" t="s">
-        <v>42</v>
-      </c>
-    </row>
-    <row r="14" ht="182" spans="1:5">
-      <c r="A14" s="7" t="s">
+      <c r="B13" s="14" t="s">
+        <v>45</v>
+      </c>
+      <c r="C13" s="17"/>
+      <c r="D13" s="14" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="14" ht="182" spans="1:6">
+      <c r="A14" s="11" t="s">
         <v>20</v>
       </c>
-      <c r="B14" s="9" t="s">
-        <v>43</v>
-      </c>
-      <c r="C14" s="9" t="s">
-        <v>44</v>
-      </c>
-    </row>
-    <row r="15" ht="26" spans="1:5">
-      <c r="A15" s="10"/>
-      <c r="B15" s="10"/>
-      <c r="C15" s="10"/>
-    </row>
-    <row r="16" ht="26" spans="1:5">
-      <c r="A16" s="7" t="s">
+      <c r="B14" s="14" t="s">
+        <v>47</v>
+      </c>
+      <c r="C14" s="17"/>
+      <c r="D14" s="14" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="15" ht="26" spans="1:6">
+      <c r="A15" s="15"/>
+      <c r="B15" s="15"/>
+      <c r="C15" s="16"/>
+      <c r="D15" s="15"/>
+    </row>
+    <row r="16" ht="26" spans="1:6">
+      <c r="A16" s="11" t="s">
         <v>23</v>
       </c>
-      <c r="B16" s="11" t="s">
+      <c r="B16" s="18" t="s">
         <v>24</v>
       </c>
-      <c r="C16" s="10"/>
-    </row>
-    <row r="17" ht="26" spans="1:3">
-      <c r="A17" s="10"/>
-      <c r="B17" s="10"/>
-      <c r="C17" s="10"/>
-    </row>
-    <row r="18" ht="409.5" spans="1:3">
-      <c r="A18" s="11" t="s">
+      <c r="C16" s="16"/>
+      <c r="D16" s="15"/>
+    </row>
+    <row r="17" ht="26" spans="1:4">
+      <c r="A17" s="15"/>
+      <c r="B17" s="15"/>
+      <c r="C17" s="16"/>
+      <c r="D17" s="15"/>
+    </row>
+    <row r="18" ht="409.5" spans="1:4">
+      <c r="A18" s="18" t="s">
         <v>25</v>
       </c>
-      <c r="B18" s="9" t="s">
-        <v>45</v>
-      </c>
-      <c r="C18" s="9" t="s">
-        <v>46</v>
+      <c r="B18" s="14" t="s">
+        <v>49</v>
+      </c>
+      <c r="C18" s="17"/>
+      <c r="D18" s="14" t="s">
+        <v>50</v>
       </c>
     </row>
   </sheetData>

</xml_diff>